<commit_message>
Updated DisplayBoard Firmware; Updated SensorBoard Firmware; Implemented basic statemachine; Changed how the CAN lib works
</commit_message>
<xml_diff>
--- a/SW/documentation/CANBus_Messages.xlsx
+++ b/SW/documentation/CANBus_Messages.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\finng\Documents\MX5-HybridDash\SW\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5BB43E-1819-4207-806E-7F060A718384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6466E3-C08E-4CAB-BA9C-7500C85CD049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-27990" yWindow="900" windowWidth="28110" windowHeight="16440" xr2:uid="{0274CC53-C38D-4913-8F75-2A01A5B072C4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
   <si>
     <t>ID</t>
   </si>
@@ -65,24 +65,12 @@
     <t>Byte 7</t>
   </si>
   <si>
-    <t>Byte 8</t>
-  </si>
-  <si>
     <t>0x01</t>
   </si>
   <si>
     <t>0x02</t>
   </si>
   <si>
-    <t>0x03</t>
-  </si>
-  <si>
-    <t>0x15</t>
-  </si>
-  <si>
-    <t>0x20</t>
-  </si>
-  <si>
     <t>Purpose</t>
   </si>
   <si>
@@ -98,27 +86,9 @@
     <t>DB</t>
   </si>
   <si>
-    <t>Requests a HW Reset</t>
-  </si>
-  <si>
     <t>8 Bit Display HW UUID</t>
   </si>
   <si>
-    <t>Requests FW Version</t>
-  </si>
-  <si>
-    <t>Major Version</t>
-  </si>
-  <si>
-    <t>Minor Version</t>
-  </si>
-  <si>
-    <t>Patch Version</t>
-  </si>
-  <si>
-    <t>Returns FW Version</t>
-  </si>
-  <si>
     <t>New Sensor Data</t>
   </si>
   <si>
@@ -143,22 +113,25 @@
     <t>Right Indicator</t>
   </si>
   <si>
-    <t>0x21</t>
-  </si>
-  <si>
-    <t>Enter Update Mode</t>
-  </si>
-  <si>
     <t>Registers itself with its HW UUID</t>
   </si>
   <si>
     <t>WTemp (0 - 255)</t>
   </si>
   <si>
-    <t>0x04</t>
-  </si>
-  <si>
     <t>Request HW UUID Register</t>
+  </si>
+  <si>
+    <t>0x10</t>
+  </si>
+  <si>
+    <t>Set ID</t>
+  </si>
+  <si>
+    <t>ID (0 - 255)</t>
+  </si>
+  <si>
+    <t>?x??</t>
   </si>
 </sst>
 </file>
@@ -629,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F12CDF6-9484-430A-ACD9-49ECAB5F74D3}">
-  <dimension ref="B2:N22"/>
+  <dimension ref="B2:M22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="37" bestFit="1" customWidth="1"/>
@@ -638,24 +611,24 @@
     <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>1</v>
@@ -678,28 +651,25 @@
       <c r="L2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="3" t="s">
+    </row>
+    <row r="3" spans="2:13" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="2:14" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
       <c r="C3" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -708,23 +678,22 @@
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-    </row>
-    <row r="4" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
@@ -733,88 +702,77 @@
       <c r="K4" s="5"/>
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-    </row>
-    <row r="5" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="5"/>
+        <v>29</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-    </row>
-    <row r="6" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>29</v>
-      </c>
       <c r="I6" s="5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="N6" s="5"/>
-    </row>
-    <row r="7" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>21</v>
-      </c>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="6"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -822,24 +780,13 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-    </row>
-    <row r="8" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>21</v>
-      </c>
+    </row>
+    <row r="8" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="6"/>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -847,40 +794,22 @@
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-    </row>
-    <row r="9" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B9" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>25</v>
-      </c>
+    </row>
+    <row r="9" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-    </row>
-    <row r="10" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -893,9 +822,8 @@
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-    </row>
-    <row r="11" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -908,9 +836,8 @@
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-    </row>
-    <row r="12" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -923,9 +850,8 @@
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-    </row>
-    <row r="13" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -938,9 +864,8 @@
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-    </row>
-    <row r="14" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
@@ -953,9 +878,8 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-    </row>
-    <row r="15" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
@@ -968,9 +892,8 @@
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-    </row>
-    <row r="16" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -983,9 +906,8 @@
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-    </row>
-    <row r="17" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -998,9 +920,8 @@
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-    </row>
-    <row r="18" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -1013,9 +934,8 @@
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-    </row>
-    <row r="19" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -1028,9 +948,8 @@
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-    </row>
-    <row r="20" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
@@ -1043,9 +962,8 @@
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-    </row>
-    <row r="21" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
@@ -1058,9 +976,8 @@
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-    </row>
-    <row r="22" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="2:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -1073,7 +990,6 @@
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M9">
@@ -1081,5 +997,6 @@
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>